<commit_message>
Client actual ordered quantities added to BOM #3
</commit_message>
<xml_diff>
--- a/Design-Files/DBS-Stepper-Module/BOM/Client BOM.xlsx
+++ b/Design-Files/DBS-Stepper-Module/BOM/Client BOM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\noelmcdermott-dbsdesign-hw\Design-Files\DBS-Stepper-Module\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,12 +14,12 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="337">
   <si>
     <t>#</t>
   </si>
@@ -1027,12 +1027,15 @@
   </si>
   <si>
     <t xml:space="preserve">Also Select optional parts  1# OEM : 0258017025.    2# AC/DC Power supply   </t>
+  </si>
+  <si>
+    <t>Client Ordered Quantity</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1105,7 +1108,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -1222,11 +1225,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1263,9 +1277,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1282,6 +1293,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1569,7 +1586,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K72"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1581,10 +1598,11 @@
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.5703125" customWidth="1"/>
+    <col min="11" max="11" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1593,11 +1611,12 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+    </row>
+    <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1627,10 +1646,13 @@
         <v>324</v>
       </c>
       <c r="K2" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="L2" s="5" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -1660,9 +1682,12 @@
       <c r="J3" s="7">
         <v>20</v>
       </c>
-      <c r="K3" s="7"/>
-    </row>
-    <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K3" s="7">
+        <v>22</v>
+      </c>
+      <c r="L3" s="7"/>
+    </row>
+    <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
         <f t="shared" ref="B4:B70" si="0">ROW(B4) - ROW($B$2)</f>
@@ -1692,9 +1717,12 @@
       <c r="J4" s="9">
         <v>2</v>
       </c>
-      <c r="K4" s="9"/>
-    </row>
-    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K4" s="9">
+        <v>4</v>
+      </c>
+      <c r="L4" s="9"/>
+    </row>
+    <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -1724,9 +1752,12 @@
       <c r="J5" s="7">
         <v>1</v>
       </c>
-      <c r="K5" s="7"/>
-    </row>
-    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K5" s="7">
+        <v>3</v>
+      </c>
+      <c r="L5" s="7"/>
+    </row>
+    <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -1756,9 +1787,12 @@
       <c r="J6" s="9">
         <v>3</v>
       </c>
-      <c r="K6" s="9"/>
-    </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K6" s="9">
+        <v>5</v>
+      </c>
+      <c r="L6" s="9"/>
+    </row>
+    <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -1788,9 +1822,12 @@
       <c r="J7" s="7">
         <v>1</v>
       </c>
-      <c r="K7" s="7"/>
-    </row>
-    <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K7" s="7">
+        <v>3</v>
+      </c>
+      <c r="L7" s="7"/>
+    </row>
+    <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
@@ -1820,9 +1857,12 @@
       <c r="J8" s="9">
         <v>3</v>
       </c>
-      <c r="K8" s="9"/>
-    </row>
-    <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K8" s="9">
+        <v>5</v>
+      </c>
+      <c r="L8" s="9"/>
+    </row>
+    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
@@ -1852,9 +1892,12 @@
       <c r="J9" s="7">
         <v>1</v>
       </c>
-      <c r="K9" s="7"/>
-    </row>
-    <row r="10" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K9" s="7">
+        <v>3</v>
+      </c>
+      <c r="L9" s="7"/>
+    </row>
+    <row r="10" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
@@ -1884,9 +1927,12 @@
       <c r="J10" s="9">
         <v>1</v>
       </c>
-      <c r="K10" s="9"/>
-    </row>
-    <row r="11" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K10" s="9">
+        <v>3</v>
+      </c>
+      <c r="L10" s="9"/>
+    </row>
+    <row r="11" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
@@ -1916,9 +1962,12 @@
       <c r="J11" s="7">
         <v>2</v>
       </c>
-      <c r="K11" s="7"/>
-    </row>
-    <row r="12" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K11" s="7">
+        <v>4</v>
+      </c>
+      <c r="L11" s="7"/>
+    </row>
+    <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
@@ -1948,9 +1997,12 @@
       <c r="J12" s="9">
         <v>2</v>
       </c>
-      <c r="K12" s="9"/>
-    </row>
-    <row r="13" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K12" s="9">
+        <v>4</v>
+      </c>
+      <c r="L12" s="9"/>
+    </row>
+    <row r="13" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -1980,9 +2032,12 @@
       <c r="J13" s="7">
         <v>2</v>
       </c>
-      <c r="K13" s="7"/>
-    </row>
-    <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K13" s="7">
+        <v>4</v>
+      </c>
+      <c r="L13" s="7"/>
+    </row>
+    <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
         <f t="shared" si="0"/>
@@ -2012,9 +2067,12 @@
       <c r="J14" s="9">
         <v>1</v>
       </c>
-      <c r="K14" s="9"/>
-    </row>
-    <row r="15" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K14" s="9">
+        <v>3</v>
+      </c>
+      <c r="L14" s="9"/>
+    </row>
+    <row r="15" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
@@ -2044,9 +2102,12 @@
       <c r="J15" s="7">
         <v>4</v>
       </c>
-      <c r="K15" s="7"/>
-    </row>
-    <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K15" s="7">
+        <v>6</v>
+      </c>
+      <c r="L15" s="7"/>
+    </row>
+    <row r="16" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
@@ -2076,9 +2137,12 @@
       <c r="J16" s="9">
         <v>4</v>
       </c>
-      <c r="K16" s="9"/>
-    </row>
-    <row r="17" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K16" s="9">
+        <v>6</v>
+      </c>
+      <c r="L16" s="9"/>
+    </row>
+    <row r="17" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
@@ -2108,9 +2172,12 @@
       <c r="J17" s="7">
         <v>2</v>
       </c>
-      <c r="K17" s="7"/>
-    </row>
-    <row r="18" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K17" s="7">
+        <v>4</v>
+      </c>
+      <c r="L17" s="7"/>
+    </row>
+    <row r="18" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -2140,9 +2207,12 @@
       <c r="J18" s="9">
         <v>1</v>
       </c>
-      <c r="K18" s="9"/>
-    </row>
-    <row r="19" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K18" s="9">
+        <v>3</v>
+      </c>
+      <c r="L18" s="9"/>
+    </row>
+    <row r="19" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
@@ -2172,9 +2242,12 @@
       <c r="J19" s="7">
         <v>1</v>
       </c>
-      <c r="K19" s="7"/>
-    </row>
-    <row r="20" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K19" s="7">
+        <v>2</v>
+      </c>
+      <c r="L19" s="7"/>
+    </row>
+    <row r="20" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
         <f t="shared" si="0"/>
@@ -2204,9 +2277,12 @@
       <c r="J20" s="9">
         <v>1</v>
       </c>
-      <c r="K20" s="9"/>
-    </row>
-    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K20" s="9">
+        <v>2</v>
+      </c>
+      <c r="L20" s="9"/>
+    </row>
+    <row r="21" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
@@ -2236,9 +2312,12 @@
       <c r="J21" s="7">
         <v>1</v>
       </c>
-      <c r="K21" s="7"/>
-    </row>
-    <row r="22" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K21" s="7">
+        <v>2</v>
+      </c>
+      <c r="L21" s="7"/>
+    </row>
+    <row r="22" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
         <f t="shared" si="0"/>
@@ -2268,9 +2347,12 @@
       <c r="J22" s="9">
         <v>1</v>
       </c>
-      <c r="K22" s="9"/>
-    </row>
-    <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K22" s="9">
+        <v>2</v>
+      </c>
+      <c r="L22" s="9"/>
+    </row>
+    <row r="23" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
@@ -2300,9 +2382,12 @@
       <c r="J23" s="7">
         <v>2</v>
       </c>
-      <c r="K23" s="7"/>
-    </row>
-    <row r="24" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K23" s="7">
+        <v>3</v>
+      </c>
+      <c r="L23" s="7"/>
+    </row>
+    <row r="24" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
         <f t="shared" si="0"/>
@@ -2332,9 +2417,12 @@
       <c r="J24" s="9">
         <v>1</v>
       </c>
-      <c r="K24" s="9"/>
-    </row>
-    <row r="25" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K24" s="9">
+        <v>1</v>
+      </c>
+      <c r="L24" s="9"/>
+    </row>
+    <row r="25" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
         <f>ROW(B25) - ROW($B$2)</f>
@@ -2364,9 +2452,12 @@
       <c r="J25" s="7">
         <v>1</v>
       </c>
-      <c r="K25" s="7"/>
-    </row>
-    <row r="26" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K25" s="7">
+        <v>1</v>
+      </c>
+      <c r="L25" s="7"/>
+    </row>
+    <row r="26" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
         <f t="shared" si="0"/>
@@ -2396,9 +2487,12 @@
       <c r="J26" s="9">
         <v>1</v>
       </c>
-      <c r="K26" s="9"/>
-    </row>
-    <row r="27" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K26" s="9">
+        <v>1</v>
+      </c>
+      <c r="L26" s="9"/>
+    </row>
+    <row r="27" spans="1:12" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
         <f>ROW(B27) - ROW($B$2)</f>
@@ -2428,9 +2522,12 @@
       <c r="J27" s="7">
         <v>1</v>
       </c>
-      <c r="K27" s="7"/>
-    </row>
-    <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K27" s="7">
+        <v>1</v>
+      </c>
+      <c r="L27" s="7"/>
+    </row>
+    <row r="28" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
         <f t="shared" si="0"/>
@@ -2460,9 +2557,12 @@
       <c r="J28" s="9">
         <v>1</v>
       </c>
-      <c r="K28" s="9"/>
-    </row>
-    <row r="29" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K28" s="9">
+        <v>1</v>
+      </c>
+      <c r="L28" s="9"/>
+    </row>
+    <row r="29" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
@@ -2492,9 +2592,12 @@
       <c r="J29" s="7">
         <v>1</v>
       </c>
-      <c r="K29" s="7"/>
-    </row>
-    <row r="30" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K29" s="7">
+        <v>1</v>
+      </c>
+      <c r="L29" s="7"/>
+    </row>
+    <row r="30" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
         <f t="shared" si="0"/>
@@ -2524,9 +2627,12 @@
       <c r="J30" s="9">
         <v>2</v>
       </c>
-      <c r="K30" s="9"/>
-    </row>
-    <row r="31" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K30" s="9">
+        <v>2</v>
+      </c>
+      <c r="L30" s="9"/>
+    </row>
+    <row r="31" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
         <f>ROW(B31) - ROW($B$2)</f>
@@ -2556,9 +2662,12 @@
       <c r="J31" s="7">
         <v>1</v>
       </c>
-      <c r="K31" s="7"/>
-    </row>
-    <row r="32" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K31" s="7">
+        <v>1</v>
+      </c>
+      <c r="L31" s="7"/>
+    </row>
+    <row r="32" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" si="0"/>
@@ -2588,9 +2697,12 @@
       <c r="J32" s="9">
         <v>1</v>
       </c>
-      <c r="K32" s="9"/>
-    </row>
-    <row r="33" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K32" s="9">
+        <v>1</v>
+      </c>
+      <c r="L32" s="9"/>
+    </row>
+    <row r="33" spans="1:12" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
         <f>ROW(B33) - ROW($B$2)</f>
@@ -2620,9 +2732,12 @@
       <c r="J33" s="7">
         <v>1</v>
       </c>
-      <c r="K33" s="7"/>
-    </row>
-    <row r="34" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K33" s="7">
+        <v>1</v>
+      </c>
+      <c r="L33" s="7"/>
+    </row>
+    <row r="34" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
         <f t="shared" si="0"/>
@@ -2652,9 +2767,12 @@
       <c r="J34" s="9">
         <v>1</v>
       </c>
-      <c r="K34" s="9"/>
-    </row>
-    <row r="35" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K34" s="9">
+        <v>1</v>
+      </c>
+      <c r="L34" s="9"/>
+    </row>
+    <row r="35" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="11">
         <f>ROW(B35) - ROW($B$2)</f>
@@ -2684,9 +2802,12 @@
       <c r="J35" s="7">
         <v>1</v>
       </c>
-      <c r="K35" s="7"/>
-    </row>
-    <row r="36" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K35" s="7">
+        <v>2</v>
+      </c>
+      <c r="L35" s="7"/>
+    </row>
+    <row r="36" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="11">
         <f t="shared" si="0"/>
@@ -2716,9 +2837,12 @@
       <c r="J36" s="9">
         <v>2</v>
       </c>
-      <c r="K36" s="9"/>
-    </row>
-    <row r="37" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K36" s="9">
+        <v>3</v>
+      </c>
+      <c r="L36" s="9"/>
+    </row>
+    <row r="37" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="11">
         <f>ROW(B37) - ROW($B$2)</f>
@@ -2748,9 +2872,12 @@
       <c r="J37" s="7">
         <v>2</v>
       </c>
-      <c r="K37" s="7"/>
-    </row>
-    <row r="38" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K37" s="7">
+        <v>3</v>
+      </c>
+      <c r="L37" s="7"/>
+    </row>
+    <row r="38" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="11">
         <f t="shared" si="0"/>
@@ -2780,9 +2907,12 @@
       <c r="J38" s="9">
         <v>2</v>
       </c>
-      <c r="K38" s="9"/>
-    </row>
-    <row r="39" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K38" s="9">
+        <v>3</v>
+      </c>
+      <c r="L38" s="9"/>
+    </row>
+    <row r="39" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="11">
         <f>ROW(B39) - ROW($B$2)</f>
@@ -2812,9 +2942,12 @@
       <c r="J39" s="7">
         <v>1</v>
       </c>
-      <c r="K39" s="7"/>
-    </row>
-    <row r="40" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K39" s="7">
+        <v>1</v>
+      </c>
+      <c r="L39" s="7"/>
+    </row>
+    <row r="40" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="11">
         <f t="shared" si="0"/>
@@ -2840,9 +2973,12 @@
       <c r="J40" s="9">
         <v>4</v>
       </c>
-      <c r="K40" s="9"/>
-    </row>
-    <row r="41" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K40" s="9">
+        <v>0</v>
+      </c>
+      <c r="L40" s="9"/>
+    </row>
+    <row r="41" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="11">
         <f>ROW(B41) - ROW($B$2)</f>
@@ -2872,9 +3008,12 @@
       <c r="J41" s="7">
         <v>2</v>
       </c>
-      <c r="K41" s="7"/>
-    </row>
-    <row r="42" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K41" s="7">
+        <v>3</v>
+      </c>
+      <c r="L41" s="7"/>
+    </row>
+    <row r="42" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="11">
         <f t="shared" si="0"/>
@@ -2902,9 +3041,12 @@
       <c r="J42" s="9">
         <v>1</v>
       </c>
-      <c r="K42" s="9"/>
-    </row>
-    <row r="43" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K42" s="9">
+        <v>2</v>
+      </c>
+      <c r="L42" s="9"/>
+    </row>
+    <row r="43" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="11">
         <f>ROW(B43) - ROW($B$2)</f>
@@ -2934,9 +3076,12 @@
       <c r="J43" s="7">
         <v>1</v>
       </c>
-      <c r="K43" s="7"/>
-    </row>
-    <row r="44" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K43" s="7">
+        <v>2</v>
+      </c>
+      <c r="L43" s="7"/>
+    </row>
+    <row r="44" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="11">
         <f t="shared" si="0"/>
@@ -2966,9 +3111,12 @@
       <c r="J44" s="9">
         <v>1</v>
       </c>
-      <c r="K44" s="9"/>
-    </row>
-    <row r="45" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K44" s="9">
+        <v>2</v>
+      </c>
+      <c r="L44" s="9"/>
+    </row>
+    <row r="45" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="11">
         <f>ROW(B45) - ROW($B$2)</f>
@@ -2998,9 +3146,12 @@
       <c r="J45" s="7">
         <v>12</v>
       </c>
-      <c r="K45" s="7"/>
-    </row>
-    <row r="46" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K45" s="7">
+        <v>14</v>
+      </c>
+      <c r="L45" s="7"/>
+    </row>
+    <row r="46" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="11">
         <f t="shared" si="0"/>
@@ -3030,9 +3181,12 @@
       <c r="J46" s="9">
         <v>2</v>
       </c>
-      <c r="K46" s="9"/>
-    </row>
-    <row r="47" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K46" s="9">
+        <v>3</v>
+      </c>
+      <c r="L46" s="9"/>
+    </row>
+    <row r="47" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="11">
         <f>ROW(B47) - ROW($B$2)</f>
@@ -3062,9 +3216,12 @@
       <c r="J47" s="7">
         <v>8</v>
       </c>
-      <c r="K47" s="7"/>
-    </row>
-    <row r="48" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K47" s="7">
+        <v>10</v>
+      </c>
+      <c r="L47" s="7"/>
+    </row>
+    <row r="48" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="11">
         <f t="shared" si="0"/>
@@ -3094,9 +3251,12 @@
       <c r="J48" s="9">
         <v>2</v>
       </c>
-      <c r="K48" s="9"/>
-    </row>
-    <row r="49" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K48" s="9">
+        <v>3</v>
+      </c>
+      <c r="L48" s="9"/>
+    </row>
+    <row r="49" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="11">
         <f>ROW(B49) - ROW($B$2)</f>
@@ -3126,9 +3286,12 @@
       <c r="J49" s="7">
         <v>4</v>
       </c>
-      <c r="K49" s="7"/>
-    </row>
-    <row r="50" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K49" s="7">
+        <v>6</v>
+      </c>
+      <c r="L49" s="7"/>
+    </row>
+    <row r="50" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="11">
         <f t="shared" si="0"/>
@@ -3158,9 +3321,12 @@
       <c r="J50" s="9">
         <v>1</v>
       </c>
-      <c r="K50" s="9"/>
-    </row>
-    <row r="51" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K50" s="9">
+        <v>2</v>
+      </c>
+      <c r="L50" s="9"/>
+    </row>
+    <row r="51" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="B51" s="11">
         <f>ROW(B51) - ROW($B$2)</f>
@@ -3190,9 +3356,12 @@
       <c r="J51" s="7">
         <v>2</v>
       </c>
-      <c r="K51" s="7"/>
-    </row>
-    <row r="52" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K51" s="7">
+        <v>3</v>
+      </c>
+      <c r="L51" s="7"/>
+    </row>
+    <row r="52" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="11">
         <f t="shared" si="0"/>
@@ -3222,9 +3391,12 @@
       <c r="J52" s="9">
         <v>2</v>
       </c>
-      <c r="K52" s="9"/>
-    </row>
-    <row r="53" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K52" s="9">
+        <v>3</v>
+      </c>
+      <c r="L52" s="9"/>
+    </row>
+    <row r="53" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
       <c r="B53" s="11">
         <f>ROW(B53) - ROW($B$2)</f>
@@ -3254,9 +3426,12 @@
       <c r="J53" s="7">
         <v>4</v>
       </c>
-      <c r="K53" s="7"/>
-    </row>
-    <row r="54" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K53" s="7">
+        <v>6</v>
+      </c>
+      <c r="L53" s="7"/>
+    </row>
+    <row r="54" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="11">
         <f t="shared" si="0"/>
@@ -3286,9 +3461,12 @@
       <c r="J54" s="9">
         <v>1</v>
       </c>
-      <c r="K54" s="9"/>
-    </row>
-    <row r="55" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K54" s="9">
+        <v>2</v>
+      </c>
+      <c r="L54" s="9"/>
+    </row>
+    <row r="55" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="11">
         <f>ROW(B55) - ROW($B$2)</f>
@@ -3318,9 +3496,12 @@
       <c r="J55" s="7">
         <v>3</v>
       </c>
-      <c r="K55" s="7"/>
-    </row>
-    <row r="56" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K55" s="7">
+        <v>4</v>
+      </c>
+      <c r="L55" s="7"/>
+    </row>
+    <row r="56" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="11">
         <f t="shared" si="0"/>
@@ -3350,9 +3531,12 @@
       <c r="J56" s="9">
         <v>2</v>
       </c>
-      <c r="K56" s="9"/>
-    </row>
-    <row r="57" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K56" s="9">
+        <v>3</v>
+      </c>
+      <c r="L56" s="9"/>
+    </row>
+    <row r="57" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="11">
         <f>ROW(B57) - ROW($B$2)</f>
@@ -3382,9 +3566,12 @@
       <c r="J57" s="7">
         <v>1</v>
       </c>
-      <c r="K57" s="7"/>
-    </row>
-    <row r="58" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K57" s="7">
+        <v>2</v>
+      </c>
+      <c r="L57" s="7"/>
+    </row>
+    <row r="58" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="11">
         <f t="shared" si="0"/>
@@ -3414,9 +3601,12 @@
       <c r="J58" s="9">
         <v>2</v>
       </c>
-      <c r="K58" s="9"/>
-    </row>
-    <row r="59" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K58" s="9">
+        <v>2</v>
+      </c>
+      <c r="L58" s="9"/>
+    </row>
+    <row r="59" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
       <c r="B59" s="11">
         <f>ROW(B59) - ROW($B$2)</f>
@@ -3446,9 +3636,12 @@
       <c r="J59" s="7">
         <v>1</v>
       </c>
-      <c r="K59" s="7"/>
-    </row>
-    <row r="60" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K59" s="7">
+        <v>1</v>
+      </c>
+      <c r="L59" s="7"/>
+    </row>
+    <row r="60" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
       <c r="B60" s="11">
         <f t="shared" si="0"/>
@@ -3478,9 +3671,12 @@
       <c r="J60" s="9">
         <v>1</v>
       </c>
-      <c r="K60" s="9"/>
-    </row>
-    <row r="61" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K60" s="9">
+        <v>1</v>
+      </c>
+      <c r="L60" s="9"/>
+    </row>
+    <row r="61" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="11">
         <f>ROW(B61) - ROW($B$2)</f>
@@ -3510,9 +3706,12 @@
       <c r="J61" s="7">
         <v>1</v>
       </c>
-      <c r="K61" s="7"/>
-    </row>
-    <row r="62" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K61" s="7">
+        <v>1</v>
+      </c>
+      <c r="L61" s="7"/>
+    </row>
+    <row r="62" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
       <c r="B62" s="11">
         <f t="shared" si="0"/>
@@ -3542,9 +3741,12 @@
       <c r="J62" s="9">
         <v>1</v>
       </c>
-      <c r="K62" s="9"/>
-    </row>
-    <row r="63" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K62" s="9">
+        <v>1</v>
+      </c>
+      <c r="L62" s="9"/>
+    </row>
+    <row r="63" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="11">
         <f>ROW(B63) - ROW($B$2)</f>
@@ -3574,9 +3776,12 @@
       <c r="J63" s="7">
         <v>1</v>
       </c>
-      <c r="K63" s="7"/>
-    </row>
-    <row r="64" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K63" s="7">
+        <v>1</v>
+      </c>
+      <c r="L63" s="7"/>
+    </row>
+    <row r="64" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
       <c r="B64" s="11">
         <f t="shared" si="0"/>
@@ -3606,9 +3811,12 @@
       <c r="J64" s="9">
         <v>1</v>
       </c>
-      <c r="K64" s="9"/>
-    </row>
-    <row r="65" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K64" s="9">
+        <v>1</v>
+      </c>
+      <c r="L64" s="9"/>
+    </row>
+    <row r="65" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
       <c r="B65" s="11">
         <f>ROW(B65) - ROW($B$2)</f>
@@ -3638,9 +3846,12 @@
       <c r="J65" s="7">
         <v>1</v>
       </c>
-      <c r="K65" s="7"/>
-    </row>
-    <row r="66" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K65" s="7">
+        <v>1</v>
+      </c>
+      <c r="L65" s="7"/>
+    </row>
+    <row r="66" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1"/>
       <c r="B66" s="11">
         <f t="shared" si="0"/>
@@ -3670,9 +3881,12 @@
       <c r="J66" s="9">
         <v>4</v>
       </c>
-      <c r="K66" s="9"/>
-    </row>
-    <row r="67" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K66" s="9">
+        <v>4</v>
+      </c>
+      <c r="L66" s="9"/>
+    </row>
+    <row r="67" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
       <c r="B67" s="11">
         <f>ROW(B67) - ROW($B$2)</f>
@@ -3702,9 +3916,12 @@
       <c r="J67" s="7">
         <v>1</v>
       </c>
-      <c r="K67" s="7"/>
-    </row>
-    <row r="68" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K67" s="7">
+        <v>1</v>
+      </c>
+      <c r="L67" s="7"/>
+    </row>
+    <row r="68" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
       <c r="B68" s="11">
         <f t="shared" si="0"/>
@@ -3734,9 +3951,12 @@
       <c r="J68" s="9">
         <v>1</v>
       </c>
-      <c r="K68" s="9"/>
-    </row>
-    <row r="69" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K68" s="9">
+        <v>1</v>
+      </c>
+      <c r="L68" s="9"/>
+    </row>
+    <row r="69" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
       <c r="B69" s="11">
         <f>ROW(B69) - ROW($B$2)</f>
@@ -3766,9 +3986,12 @@
       <c r="J69" s="7">
         <v>1</v>
       </c>
-      <c r="K69" s="7"/>
-    </row>
-    <row r="70" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K69" s="7">
+        <v>1</v>
+      </c>
+      <c r="L69" s="7"/>
+    </row>
+    <row r="70" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1"/>
       <c r="B70" s="11">
         <f t="shared" si="0"/>
@@ -3798,10 +4021,13 @@
       <c r="J70" s="9">
         <v>2</v>
       </c>
-      <c r="K70" s="9"/>
-    </row>
-    <row r="71" spans="1:11" ht="78.75" x14ac:dyDescent="0.25">
-      <c r="B71" s="15">
+      <c r="K70" s="9">
+        <v>2</v>
+      </c>
+      <c r="L70" s="9"/>
+    </row>
+    <row r="71" spans="1:12" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="B71" s="14">
         <f t="shared" ref="B71:B72" si="1">ROW(B71) - ROW($B$7)</f>
         <v>64</v>
       </c>
@@ -3827,40 +4053,46 @@
       <c r="J71" s="9">
         <v>1</v>
       </c>
-      <c r="K71" s="16" t="s">
+      <c r="K71" s="21" t="s">
+        <v>327</v>
+      </c>
+      <c r="L71" s="15" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B72" s="17">
+    <row r="72" spans="1:12" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B72" s="16">
         <f t="shared" si="1"/>
         <v>65</v>
       </c>
-      <c r="C72" s="18" t="s">
+      <c r="C72" s="17" t="s">
         <v>329</v>
       </c>
-      <c r="D72" s="19" t="s">
+      <c r="D72" s="18" t="s">
         <v>327</v>
       </c>
-      <c r="E72" s="19" t="s">
+      <c r="E72" s="18" t="s">
         <v>333</v>
       </c>
-      <c r="F72" s="19" t="s">
+      <c r="F72" s="18" t="s">
         <v>327</v>
       </c>
-      <c r="G72" s="19" t="s">
+      <c r="G72" s="18" t="s">
         <v>334</v>
       </c>
-      <c r="H72" s="19"/>
-      <c r="I72" s="19"/>
-      <c r="J72" s="19">
-        <v>1</v>
-      </c>
-      <c r="K72" s="20"/>
+      <c r="H72" s="18"/>
+      <c r="I72" s="18"/>
+      <c r="J72" s="18">
+        <v>1</v>
+      </c>
+      <c r="K72" s="9">
+        <v>1</v>
+      </c>
+      <c r="L72" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I1:L1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>